<commit_message>
penambahan filter untuk hardware sesuai ID gatenya
</commit_message>
<xml_diff>
--- a/Database-app.xlsx
+++ b/Database-app.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="264" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="190">
   <si>
     <t>ID_Gate</t>
   </si>
@@ -190,12 +190,18 @@
     <t>Membaca plat nomor</t>
   </si>
   <si>
+    <t>FAIL</t>
+  </si>
+  <si>
     <t>LPR_A01</t>
   </si>
   <si>
     <t>Kamera LPR A01</t>
   </si>
   <si>
+    <t>PASS</t>
+  </si>
+  <si>
     <t>OCR_A02</t>
   </si>
   <si>
@@ -211,7 +217,7 @@
     <t>Kamera OCR A01</t>
   </si>
   <si>
-    <t>CROSS_ARROW_A02</t>
+    <t>CROSSARROW_A02</t>
   </si>
   <si>
     <t>Cross Arrow A02</t>
@@ -223,12 +229,45 @@
     <t>Informasi jalur active / nonactive</t>
   </si>
   <si>
-    <t>CROSS_ARROW_A01</t>
+    <t>CROSSARROW_A01</t>
   </si>
   <si>
     <t>Cross Arrow A01</t>
   </si>
   <si>
+    <t>WARNING</t>
+  </si>
+  <si>
+    <t>LEDMatrix_A02</t>
+  </si>
+  <si>
+    <t>LEDMatrix_A01</t>
+  </si>
+  <si>
+    <t>TrafficLight_A02</t>
+  </si>
+  <si>
+    <t>TrafficLight_A01</t>
+  </si>
+  <si>
+    <t>BarrierGate_A02</t>
+  </si>
+  <si>
+    <t>Barrier Gate</t>
+  </si>
+  <si>
+    <t>BarrierGate_A01</t>
+  </si>
+  <si>
+    <t>OBS_A02</t>
+  </si>
+  <si>
+    <t>Sensor</t>
+  </si>
+  <si>
+    <t>OBS_A01</t>
+  </si>
+  <si>
     <t>LPR_C01</t>
   </si>
   <si>
@@ -259,12 +298,6 @@
     <t>Watermark</t>
   </si>
   <si>
-    <t>Barrier Gate</t>
-  </si>
-  <si>
-    <t>PASS</t>
-  </si>
-  <si>
     <t>test data</t>
   </si>
   <si>
@@ -283,9 +316,6 @@
     <t>Petugas: Adam | Gate: C01 | Waktu: Tue Apr 21 2026 11:40:12 GMT+0700 (Waktu Indonesia Barat)</t>
   </si>
   <si>
-    <t>FAIL</t>
-  </si>
-  <si>
     <t>test sync</t>
   </si>
   <si>
@@ -293,9 +323,6 @@
   </si>
   <si>
     <t>Petugas: Adam | Gate: C01 | Lokasi: Pelabuhan | Waktu: Tue Apr 21 2026 11:58:37 GMT+0700 (Waktu Indonesia Barat)</t>
-  </si>
-  <si>
-    <t>WARNING</t>
   </si>
   <si>
     <t>test multiple inputt</t>
@@ -433,6 +460,66 @@
     <t>Petugas: Adam | Gate: C01 | Lokasi: Pelabuhan | Waktu: Wed Apr 22 2026 16:01:22 GMT+0700 (Western Indonesia Time)</t>
   </si>
   <si>
+    <t>test ea</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1ZwGR6q7U63nezaHQ_ou768ho-9DPTShm/view?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>Petugas: Adam | Gate: C01 | Lokasi: Pelabuhan | Waktu: Wed Apr 22 2026 16:21:29 GMT+0700 (Western Indonesia Time)</t>
+  </si>
+  <si>
+    <t>Petugas: Zaky | Gate: A01 | Lokasi: Kawasan | Waktu: Wed Apr 22 2026 16:32:53 GMT+0700 (Western Indonesia Time)</t>
+  </si>
+  <si>
+    <t>Pwcah</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1pdU2HRq6HGzXNJvTZ4ruhUSKaG1zJE_N/view?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>Petugas: Zaky | Gate: A02 | Lokasi: Kawasan | Waktu: Wed Apr 22 2026 16:45:31 GMT+0700 (Western Indonesia Time)</t>
+  </si>
+  <si>
+    <t>Kotor</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1Yk0wQh2noQIVoY-iFH0S-JecLgUgX4JY/view?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>Petugas: Zaky | Gate: A01 | Lokasi: Kawasan | Waktu: Wed Apr 22 2026 16:46:53 GMT+0700 (Western Indonesia Time)</t>
+  </si>
+  <si>
+    <t>normal</t>
+  </si>
+  <si>
+    <t>Petugas: Zaky | Gate: A01 | Lokasi: Kawasan | Waktu: Wed Apr 22 2026 16:47:47 GMT+0700 (Western Indonesia Time)</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1g1i7k8yNND_EfdD2x1Z2pyTxApXm35Vq/view?usp=drivesdk ,https://drive.google.com/file/d/1X6jV2fcDlQ_QPH7qKyaZRRrrmCmmsggj/view?usp=drivesdk ,https://drive.google.com/file/d/1trqAjVRcoHwtTj5ojfwNf3ZVnXcYLT_3/view?usp=drivesdk ,https://drive.google.com/file/d/1pxv66ozxCRQJlbomgkkuFFBs72Dz8P1s/view?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>Petugas: Zaky | Gate: A02 | Lokasi: Kawasan | Waktu: Thu Apr 23 2026 16:41:06 GMT+0700 (Western Indonesia Time)</t>
+  </si>
+  <si>
+    <t>test berkedip</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1RCYg3YoBQUWmRjoOXA4OMSoSot6HE23I/view?usp=drivesdk ,https://drive.google.com/file/d/15fERfFNQFIOcJC8HAP5k0jhjHkE5g0z5/view?usp=drivesdk ,https://drive.google.com/file/d/1iKl9p5OnmZ4ciOt0A85tToMBwmFs64zI/view?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>Petugas: Zaky | Gate: A01 | Lokasi: Kawasan | Waktu: Fri Apr 24 2026 08:53:23 GMT+0700 (Western Indonesia Time)</t>
+  </si>
+  <si>
+    <t>test bengkok</t>
+  </si>
+  <si>
+    <t>https://drive.google.com/file/d/1pw1s2u29CuluDr21ItKrHrGt9fAQmdM8/view?usp=drivesdk</t>
+  </si>
+  <si>
+    <t>Petugas: Zaky | Gate: A02 | Lokasi: Kawasan | Waktu: Fri Apr 24 2026 08:54:24 GMT+0700 (Western Indonesia Time)</t>
+  </si>
+  <si>
     <t>ID_Tiket</t>
   </si>
   <si>
@@ -505,6 +592,31 @@
   </si>
   <si>
     <t>Updated by: Adam | Gate: C01 | Tiket: MT-20260422140323 | Waktu: Wed Apr 22 2026 16:02:30 GMT+0700 (Western Indonesia Time)</t>
+  </si>
+  <si>
+    <t>TKT-20260422164531-220</t>
+  </si>
+  <si>
+    <t>Pwcah
+Update: Pecah</t>
+  </si>
+  <si>
+    <t>Pergantian kaca</t>
+  </si>
+  <si>
+    <t>Updated by: Zaky | Gate: A02 | Tiket: TKT-20260422164531-220 | Waktu: Wed Apr 22 2026 16:49:07 GMT+0700 (Western Indonesia Time)</t>
+  </si>
+  <si>
+    <t>TKT-20260422164653-770</t>
+  </si>
+  <si>
+    <t>TKT-20260423164106-577</t>
+  </si>
+  <si>
+    <t>TKT-20260424085323-67</t>
+  </si>
+  <si>
+    <t>TKT-20260424085424-263</t>
   </si>
   <si>
     <t>ID_Part</t>
@@ -5350,7 +5462,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="18.13"/>
     <col customWidth="1" min="2" max="2" width="14.0"/>
-    <col customWidth="1" min="4" max="4" width="20.88"/>
+    <col customWidth="1" min="4" max="4" width="24.75"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5369,6 +5481,12 @@
       <c r="E1" s="1" t="s">
         <v>45</v>
       </c>
+      <c r="F1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>0</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
@@ -5383,14 +5501,23 @@
       <c r="D2" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E2" s="1"/>
+      <c r="E2" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" s="1" t="str">
+        <f t="shared" ref="G2:G15" si="1">RIGHT(A2,LEN(A2) - (FIND("_",A2)))</f>
+        <v>A02</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>55</v>
@@ -5398,69 +5525,263 @@
       <c r="D3" s="1" t="s">
         <v>56</v>
       </c>
+      <c r="E3" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" s="1" t="str">
+        <f t="shared" si="1"/>
+        <v>A01</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>55</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G4" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A02</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>55</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>61</v>
+        <v>63</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G5" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A01</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>67</v>
+        <v>69</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G6" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A02</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="D7" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>66</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>67</v>
+      <c r="E7" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A01</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G8" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A02</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G9" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A01</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G10" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A02</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G11" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A01</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G12" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A02</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G13" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A01</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G14" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A02</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G15" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>A01</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="s">
-        <v>70</v>
+        <v>83</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>55</v>
@@ -5468,8 +5789,14 @@
       <c r="D25" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="1" t="b">
-        <v>1</v>
+      <c r="E25" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -5486,10 +5813,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>72</v>
+        <v>85</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -5498,22 +5825,22 @@
         <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>77</v>
+        <v>90</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>78</v>
+        <v>91</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2">
@@ -5527,19 +5854,19 @@
         <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="F2" s="1" t="s">
         <v>46</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>82</v>
+        <v>93</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3">
@@ -5553,22 +5880,22 @@
         <v>28</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="F3" s="1" t="s">
         <v>46</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="H3" s="6" t="s">
-        <v>86</v>
+        <v>97</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>87</v>
+        <v>98</v>
       </c>
     </row>
     <row r="4">
@@ -5582,22 +5909,22 @@
         <v>28</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="F4" s="1" t="s">
         <v>46</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="H4" s="6" t="s">
-        <v>90</v>
+        <v>100</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>91</v>
+        <v>101</v>
       </c>
     </row>
     <row r="5">
@@ -5611,22 +5938,22 @@
         <v>5</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>46</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6">
@@ -5640,22 +5967,22 @@
         <v>13</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>46</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="H6" s="7" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
     </row>
     <row r="7">
@@ -5669,22 +5996,22 @@
         <v>5</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="F7" s="1" t="s">
         <v>46</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
     </row>
     <row r="8">
@@ -5698,22 +6025,22 @@
         <v>5</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="F8" s="1" t="s">
         <v>46</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
     </row>
     <row r="9">
@@ -5727,22 +6054,22 @@
         <v>13</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>88</v>
+        <v>57</v>
       </c>
       <c r="F9" s="1" t="s">
         <v>48</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10">
@@ -5756,22 +6083,22 @@
         <v>28</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>92</v>
+        <v>72</v>
       </c>
       <c r="F10" s="1" t="s">
         <v>46</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11">
@@ -5785,44 +6112,243 @@
         <v>28</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>81</v>
+        <v>60</v>
       </c>
       <c r="F11" s="1" t="s">
         <v>46</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
     </row>
     <row r="12">
-      <c r="E12" s="3"/>
+      <c r="A12" s="4">
+        <v>46134.68159400463</v>
+      </c>
+      <c r="B12" s="5">
+        <v>46134.0</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>84</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="G12" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>124</v>
+      </c>
+      <c r="K12" s="1" t="s">
+        <v>125</v>
+      </c>
     </row>
     <row r="13">
-      <c r="E13" s="3"/>
+      <c r="A13" s="4">
+        <v>46134.68950956019</v>
+      </c>
+      <c r="B13" s="5">
+        <v>46134.0</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="K13" s="1" t="s">
+        <v>126</v>
+      </c>
     </row>
     <row r="14">
-      <c r="E14" s="3"/>
+      <c r="A14" s="4">
+        <v>46134.69828078704</v>
+      </c>
+      <c r="B14" s="5">
+        <v>46134.0</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="H14" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>129</v>
+      </c>
     </row>
     <row r="15">
-      <c r="E15" s="3"/>
+      <c r="A15" s="4">
+        <v>46134.699227199075</v>
+      </c>
+      <c r="B15" s="5">
+        <v>46134.0</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="K15" s="1" t="s">
+        <v>132</v>
+      </c>
     </row>
     <row r="16">
-      <c r="E16" s="3"/>
+      <c r="A16" s="4">
+        <v>46134.69985012732</v>
+      </c>
+      <c r="B16" s="5">
+        <v>46134.0</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G16" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="K16" s="1" t="s">
+        <v>134</v>
+      </c>
     </row>
     <row r="17">
-      <c r="E17" s="3"/>
+      <c r="A17" s="4">
+        <v>46135.69521523148</v>
+      </c>
+      <c r="B17" s="5">
+        <v>46135.0</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G17" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="K17" s="1" t="s">
+        <v>136</v>
+      </c>
     </row>
     <row r="18">
-      <c r="E18" s="3"/>
+      <c r="A18" s="4">
+        <v>46136.37040626157</v>
+      </c>
+      <c r="B18" s="5">
+        <v>46136.0</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G18" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="H18" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="K18" s="1" t="s">
+        <v>139</v>
+      </c>
     </row>
     <row r="19">
-      <c r="E19" s="3"/>
+      <c r="A19" s="4">
+        <v>46136.37111162037</v>
+      </c>
+      <c r="B19" s="5">
+        <v>46136.0</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>142</v>
+      </c>
     </row>
     <row r="20">
       <c r="E20" s="3"/>
@@ -8778,8 +9304,12 @@
     <hyperlink r:id="rId2" ref="H4"/>
     <hyperlink r:id="rId3" ref="H6"/>
     <hyperlink r:id="rId4" ref="H7"/>
+    <hyperlink r:id="rId5" ref="H12"/>
+    <hyperlink r:id="rId6" ref="H14"/>
+    <hyperlink r:id="rId7" ref="H15"/>
+    <hyperlink r:id="rId8" ref="H19"/>
   </hyperlinks>
-  <drawing r:id="rId5"/>
+  <drawing r:id="rId9"/>
 </worksheet>
 </file>
 
@@ -8792,10 +9322,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>143</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>115</v>
+        <v>144</v>
       </c>
       <c r="C1" s="1" t="s">
         <v>0</v>
@@ -8804,27 +9334,27 @@
         <v>49</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>116</v>
+        <v>145</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>117</v>
+        <v>146</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>118</v>
+        <v>147</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>119</v>
+        <v>148</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>120</v>
+        <v>149</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>79</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>121</v>
+        <v>150</v>
       </c>
       <c r="B2" s="5">
         <v>46133.0</v>
@@ -8833,30 +9363,30 @@
         <v>5</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>84</v>
+        <v>95</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>122</v>
+        <v>151</v>
       </c>
       <c r="F2" s="5">
         <v>46135.0</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>123</v>
+        <v>152</v>
       </c>
       <c r="H2" s="1" t="s">
         <v>46</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>124</v>
+        <v>153</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>125</v>
+        <v>154</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>126</v>
+        <v>155</v>
       </c>
       <c r="B3" s="5">
         <v>46134.0</v>
@@ -8865,24 +9395,24 @@
         <v>34</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>127</v>
+        <v>156</v>
       </c>
       <c r="H3" s="1" t="s">
         <v>48</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>128</v>
+        <v>157</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>129</v>
+        <v>158</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>130</v>
+        <v>159</v>
       </c>
       <c r="B4" s="5">
         <v>46134.0</v>
@@ -8891,24 +9421,24 @@
         <v>13</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>131</v>
+        <v>160</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>48</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>132</v>
+        <v>161</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>133</v>
+        <v>162</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>134</v>
+        <v>163</v>
       </c>
       <c r="B5" s="5">
         <v>46134.0</v>
@@ -8917,25 +9447,137 @@
         <v>28</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>71</v>
+        <v>84</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>135</v>
+        <v>164</v>
       </c>
       <c r="F5" s="5">
         <v>46134.0</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>136</v>
+        <v>165</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>46</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>124</v>
+        <v>153</v>
       </c>
       <c r="J5" s="1" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B6" s="5">
+        <v>46134.0</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="F6" s="5">
+        <v>46134.0</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="I6" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B7" s="5">
+        <v>46134.0</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="I7" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="s">
+        <v>172</v>
+      </c>
+      <c r="B8" s="5">
+        <v>46135.0</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B9" s="5">
+        <v>46136.0</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>137</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="B10" s="5">
+        <v>46136.0</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>140</v>
+      </c>
+      <c r="I10" s="1" t="s">
+        <v>157</v>
       </c>
     </row>
   </sheetData>
@@ -8952,16 +9594,16 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>138</v>
+        <v>175</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>139</v>
+        <v>176</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>140</v>
+        <v>177</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>141</v>
+        <v>178</v>
       </c>
     </row>
   </sheetData>
@@ -8990,18 +9632,18 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="8" t="s">
-        <v>142</v>
+        <v>179</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="9" t="s">
-        <v>143</v>
+        <v>180</v>
       </c>
       <c r="B3" s="10"/>
     </row>
     <row r="4">
       <c r="A4" s="11" t="s">
-        <v>144</v>
+        <v>181</v>
       </c>
       <c r="B4" s="12">
         <v>46133.0</v>
@@ -9009,7 +9651,7 @@
     </row>
     <row r="5">
       <c r="A5" s="11" t="s">
-        <v>145</v>
+        <v>182</v>
       </c>
       <c r="B5" s="12">
         <v>46142.0</v>
@@ -9025,34 +9667,34 @@
     </row>
     <row r="9">
       <c r="A9" s="14" t="s">
-        <v>146</v>
+        <v>183</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>147</v>
+        <v>184</v>
       </c>
       <c r="C9" s="14" t="s">
-        <v>148</v>
+        <v>185</v>
       </c>
       <c r="D9" s="14" t="s">
-        <v>74</v>
+        <v>87</v>
       </c>
       <c r="E9" s="14" t="s">
-        <v>75</v>
+        <v>88</v>
       </c>
       <c r="F9" s="14" t="s">
-        <v>76</v>
+        <v>89</v>
       </c>
       <c r="H9" s="15" t="s">
-        <v>149</v>
+        <v>186</v>
       </c>
       <c r="I9" s="16" t="s">
-        <v>150</v>
+        <v>187</v>
       </c>
       <c r="J9" s="17" t="s">
-        <v>151</v>
+        <v>188</v>
       </c>
       <c r="K9" s="16" t="s">
-        <v>152</v>
+        <v>189</v>
       </c>
     </row>
     <row r="10">

</xml_diff>